<commit_message>
Added `Devoid` cards for sort testing.
</commit_message>
<xml_diff>
--- a/test/fixture/snapshot/cli/export-excel/by-type.xlsx
+++ b/test/fixture/snapshot/cli/export-excel/by-type.xlsx
@@ -1921,11 +1921,64 @@
       <text>
         <r>
           <t xml:space="preserve">Border: black
+Finish: normal
+Keywords:
+➤ Devoid</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Devoid (This card has no color.)
+Exile target nonland permanent. You may cast that card for as long as it remains exiled, and you may spend colorless mana as though it were mana of any color to cast that spell.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">➤ 2 generic
+➤ 1 white
+➤ 1 black</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D73" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Border: black
+Finish: normal
+Keywords:
+➤ Devoid</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E73" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Devoid (This card has no color.)
+Counter target spell unless its controller pays {1}. You create a 1/1 colorless Eldrazi Scion creature token. It has "Sacrifice this token: Add {C}." ({C} represents colorless mana.)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J73" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">➤ 2 generic
+➤ 1 blue</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D74" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Border: black
 Finish: normal</t>
         </r>
       </text>
     </comment>
-    <comment ref="E72" authorId="0">
+    <comment ref="E74" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Choose one. If you control a commander as you cast this spell, you may choose both instead.
@@ -1934,7 +1987,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J72" authorId="0">
+    <comment ref="J74" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 3 generic
@@ -1942,7 +1995,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D73" authorId="0">
+    <comment ref="D75" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -1950,14 +2003,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E73" authorId="0">
+    <comment ref="E75" authorId="0">
       <text>
         <r>
           <t>Exile target nonland permanent. You lose 3 life.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J73" authorId="0">
+    <comment ref="J75" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 generic
@@ -1966,7 +2019,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D74" authorId="0">
+    <comment ref="D76" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -1974,14 +2027,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E74" authorId="0">
+    <comment ref="E76" authorId="0">
       <text>
         <r>
           <t>Destroy target permanent an opponent controls. Its controller may search their library for a basic land card, put it onto the battlefield, then shuffle.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J74" authorId="0">
+    <comment ref="J76" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 black
@@ -1989,7 +2042,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D75" authorId="0">
+    <comment ref="D77" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -1999,14 +2052,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E75" authorId="0">
+    <comment ref="E77" authorId="0">
       <text>
         <r>
           <t>Destroy target nonland permanent. Proliferate. (Choose any number of permanents and/or players, then give each another counter of each kind already there.)</t>
         </r>
       </text>
     </comment>
-    <comment ref="J75" authorId="0">
+    <comment ref="J77" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 2 generic
@@ -2015,7 +2068,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D76" authorId="0">
+    <comment ref="D78" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2023,14 +2076,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E76" authorId="0">
+    <comment ref="E78" authorId="0">
       <text>
         <r>
           <t>Up to one target creature gets -X/-X until end of turn. If X is 5 or more, return a creature card with mana value X or less from your graveyard to the battlefield tapped.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J76" authorId="0">
+    <comment ref="J78" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1× 𝗫 generic
@@ -2038,7 +2091,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D77" authorId="0">
+    <comment ref="D79" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Game Changer
@@ -2049,7 +2102,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E77" authorId="0">
+    <comment ref="E79" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Return target nonland permanent you don't control to its owner's hand.
@@ -2057,7 +2110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J77" authorId="0">
+    <comment ref="J79" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 generic
@@ -2065,7 +2118,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D78" authorId="0">
+    <comment ref="D80" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: borderless
@@ -2073,7 +2126,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E78" authorId="0">
+    <comment ref="E80" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">If you control a commander, you may cast this spell without paying its mana cost.
@@ -2081,7 +2134,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J78" authorId="0">
+    <comment ref="J80" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 3 generic
@@ -2089,7 +2142,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D79" authorId="0">
+    <comment ref="D81" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2097,7 +2150,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E79" authorId="0">
+    <comment ref="E81" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Choose one —
@@ -2106,7 +2159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J79" authorId="0">
+    <comment ref="J81" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 blue
@@ -2114,7 +2167,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D80" authorId="0">
+    <comment ref="D82" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2124,7 +2177,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E80" authorId="0">
+    <comment ref="E82" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Exile target creature you control, then return it to the battlefield under its owner's control.
@@ -2132,14 +2185,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="J80" authorId="0">
+    <comment ref="J82" authorId="0">
       <text>
         <r>
           <t>➤ 1 white</t>
         </r>
       </text>
     </comment>
-    <comment ref="D81" authorId="0">
+    <comment ref="D83" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Game Changer
@@ -2148,7 +2201,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E81" authorId="0">
+    <comment ref="E83" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">If you control a commander, you may cast this spell without paying its mana cost.
@@ -2156,7 +2209,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J81" authorId="0">
+    <comment ref="J83" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 2 generic
@@ -2164,7 +2217,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D82" authorId="0">
+    <comment ref="D84" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2172,7 +2225,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E82" authorId="0">
+    <comment ref="E84" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">If it's not your turn, you may exile a blue card from your hand rather than pay this spell's mana cost.
@@ -2180,7 +2233,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J82" authorId="0">
+    <comment ref="J84" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 generic
@@ -2188,7 +2241,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D83" authorId="0">
+    <comment ref="D85" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2196,7 +2249,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E83" authorId="0">
+    <comment ref="E85" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Destroy target creature that was dealt damage this turn.
@@ -2204,14 +2257,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="J83" authorId="0">
+    <comment ref="J85" authorId="0">
       <text>
         <r>
           <t>➤ 1 black</t>
         </r>
       </text>
     </comment>
-    <comment ref="D84" authorId="0">
+    <comment ref="D86" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2219,7 +2272,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E84" authorId="0">
+    <comment ref="E86" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped unless a player has 13 or less life.
@@ -2227,14 +2280,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="C85" authorId="0">
+    <comment ref="C87" authorId="0">
       <text>
         <r>
           <t>Group: external</t>
         </r>
       </text>
     </comment>
-    <comment ref="D85" authorId="0">
+    <comment ref="D87" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2242,7 +2295,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E85" authorId="0">
+    <comment ref="E87" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped unless a player has 13 or less life.
@@ -2250,7 +2303,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D86" authorId="0">
+    <comment ref="D88" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2260,7 +2313,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E86" authorId="0">
+    <comment ref="E88" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped unless you control a legendary green creature.
@@ -2270,7 +2323,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D87" authorId="0">
+    <comment ref="D89" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2278,7 +2331,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E87" authorId="0">
+    <comment ref="E89" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped.
@@ -2286,7 +2339,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D88" authorId="0">
+    <comment ref="D90" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2294,7 +2347,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E88" authorId="0">
+    <comment ref="E90" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped unless you have two or more opponents.
@@ -2302,7 +2355,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D89" authorId="0">
+    <comment ref="D91" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2310,14 +2363,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E89" authorId="0">
+    <comment ref="E91" authorId="0">
       <text>
         <r>
           <t>{T}: Add one mana of any color in your commander's color identity.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D90" authorId="0">
+    <comment ref="D92" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2325,7 +2378,23 @@
         </r>
       </text>
     </comment>
-    <comment ref="E90" authorId="0">
+    <comment ref="E92" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">{T}: Add {C}. ({C} represents colorless mana.)
+{T}, Pay 1 life: Add one mana of any color. Spend this mana only to cast a spell with devoid.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D93" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Border: black
+Finish: normal</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E93" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped.
@@ -2333,7 +2402,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D91" authorId="0">
+    <comment ref="D94" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2341,7 +2410,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E91" authorId="0">
+    <comment ref="E94" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">As this land enters, you may reveal a Soldier card from your hand. This land enters tapped unless you revealed a Soldier card this way or you control a Soldier.
@@ -2350,7 +2419,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D92" authorId="0">
+    <comment ref="D95" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2358,7 +2427,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E92" authorId="0">
+    <comment ref="E95" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">{T}: Add {C}.
@@ -2366,7 +2435,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D93" authorId="0">
+    <comment ref="D96" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2376,7 +2445,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E93" authorId="0">
+    <comment ref="E96" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">({T}: Add {W}, {B}, or {G}.)
@@ -2385,7 +2454,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D94" authorId="0">
+    <comment ref="D97" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2393,14 +2462,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E94" authorId="0">
+    <comment ref="E97" authorId="0">
       <text>
         <r>
           <t>{T}, Pay 1 life: Add one mana of any color.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D95" authorId="0">
+    <comment ref="D98" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2410,7 +2479,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E95" authorId="0">
+    <comment ref="E98" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped.
@@ -2418,7 +2487,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D96" authorId="0">
+    <comment ref="D99" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2426,14 +2495,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E96" authorId="0">
+    <comment ref="E99" authorId="0">
       <text>
         <r>
           <t>{T}, Pay 1 life, Sacrifice this land: Search your library for a basic land card, put it onto the battlefield, then shuffle.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D97" authorId="0">
+    <comment ref="D100" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: borderless
@@ -2443,7 +2512,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E97" authorId="0">
+    <comment ref="E100" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">({T}: Add {W}, {U}, or {B}.)
@@ -2452,7 +2521,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D98" authorId="0">
+    <comment ref="D101" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2460,7 +2529,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E98" authorId="0">
+    <comment ref="E101" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped unless you have two or more opponents.
@@ -2468,7 +2537,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D99" authorId="0">
+    <comment ref="D102" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2478,7 +2547,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E99" authorId="0">
+    <comment ref="E102" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">({T}: Add {G}, {W}, or {U}.)
@@ -2487,7 +2556,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D100" authorId="0">
+    <comment ref="D103" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2497,7 +2566,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E100" authorId="0">
+    <comment ref="E103" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped.
@@ -2506,7 +2575,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D101" authorId="0">
+    <comment ref="D104" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2516,7 +2585,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E101" authorId="0">
+    <comment ref="E104" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">({T}: Add {U} or {B}.)
@@ -2525,7 +2594,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D102" authorId="0">
+    <comment ref="D105" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2533,7 +2602,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E102" authorId="0">
+    <comment ref="E105" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">This land enters tapped unless you have two or more opponents.
@@ -2541,7 +2610,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D103" authorId="0">
+    <comment ref="D106" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2551,7 +2620,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E103" authorId="0">
+    <comment ref="E106" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">({T}: Add {B}, {G}, or {U}.)
@@ -2560,7 +2629,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D104" authorId="0">
+    <comment ref="D107" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2570,7 +2639,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E104" authorId="0">
+    <comment ref="E107" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">{T}: Add {G}.
@@ -2578,7 +2647,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D105" authorId="0">
+    <comment ref="D108" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2588,7 +2657,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E105" authorId="0">
+    <comment ref="E108" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">{T}: Add {W}.
@@ -2596,7 +2665,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D106" authorId="0">
+    <comment ref="D109" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2604,14 +2673,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E106" authorId="0">
+    <comment ref="E109" authorId="0">
       <text>
         <r>
           <t>Each land is a Forest in addition to its other land types.</t>
         </r>
       </text>
     </comment>
-    <comment ref="D107" authorId="0">
+    <comment ref="D110" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2619,7 +2688,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E107" authorId="0">
+    <comment ref="E110" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">(As this Saga enters and after your draw step, add a lore counter. Sacrifice after III.)
@@ -2629,7 +2698,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D108" authorId="0">
+    <comment ref="D111" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2637,7 +2706,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E108" authorId="0">
+    <comment ref="E111" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">({T}: Add {R} or {W}.)
@@ -2645,7 +2714,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D109" authorId="0">
+    <comment ref="D112" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Loyalty: 5
@@ -2654,7 +2723,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E109" authorId="0">
+    <comment ref="E112" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Creatures you control have vigilance.
@@ -2663,7 +2732,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J109" authorId="0">
+    <comment ref="J112" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 2 generic
@@ -2672,7 +2741,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D110" authorId="0">
+    <comment ref="D113" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Loyalty: 3
@@ -2681,7 +2750,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E110" authorId="0">
+    <comment ref="E113" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">+1: Draw a card, then put a card from your hand on top of your library.
@@ -2691,7 +2760,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J110" authorId="0">
+    <comment ref="J113" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 white
@@ -2700,7 +2769,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D111" authorId="0">
+    <comment ref="D114" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Loyalty: 5
@@ -2711,7 +2780,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E111" authorId="0">
+    <comment ref="E114" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Spells and abilities your opponents control can't cause their controller to search their library.
@@ -2719,7 +2788,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J111" authorId="0">
+    <comment ref="J114" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 generic
@@ -2727,7 +2796,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D112" authorId="0">
+    <comment ref="D115" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Loyalty: 5
@@ -2736,7 +2805,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E112" authorId="0">
+    <comment ref="E115" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Activated abilities of artifacts your opponents control can't be activated.
@@ -2745,14 +2814,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="J112" authorId="0">
+    <comment ref="J115" authorId="0">
       <text>
         <r>
           <t>➤ 4 generic</t>
         </r>
       </text>
     </comment>
-    <comment ref="D113" authorId="0">
+    <comment ref="D116" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Loyalty: 5
@@ -2762,7 +2831,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E113" authorId="0">
+    <comment ref="E116" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Each opponent can't draw more than one card each turn.
@@ -2770,7 +2839,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J113" authorId="0">
+    <comment ref="J116" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 generic
@@ -2778,7 +2847,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D114" authorId="0">
+    <comment ref="D117" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Loyalty: 4
@@ -2787,7 +2856,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E114" authorId="0">
+    <comment ref="E117" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">+1: Tap target permanent. It doesn't untap during its controller's next untap step.
@@ -2796,7 +2865,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J114" authorId="0">
+    <comment ref="J117" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 3 generic
@@ -2804,7 +2873,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D115" authorId="0">
+    <comment ref="D118" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2812,7 +2881,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E115" authorId="0">
+    <comment ref="E118" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Return from your graveyard to the battlefield any number of target creature cards that each have a different mana value X or less.
@@ -2822,7 +2891,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J115" authorId="0">
+    <comment ref="J118" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1× 𝗫 generic
@@ -2832,14 +2901,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="C116" authorId="0">
+    <comment ref="C119" authorId="0">
       <text>
         <r>
           <t>Group: external</t>
         </r>
       </text>
     </comment>
-    <comment ref="D116" authorId="0">
+    <comment ref="D119" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2847,7 +2916,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E116" authorId="0">
+    <comment ref="E119" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Return from your graveyard to the battlefield any number of target creature cards that each have a different mana value X or less.
@@ -2857,7 +2926,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J116" authorId="0">
+    <comment ref="J119" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1× 𝗫 generic
@@ -2867,7 +2936,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D117" authorId="0">
+    <comment ref="D120" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2877,7 +2946,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E117" authorId="0">
+    <comment ref="E120" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Create a 3/3 green Centaur creature token.
@@ -2888,7 +2957,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J117" authorId="0">
+    <comment ref="J120" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 3 generic
@@ -2898,7 +2967,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D118" authorId="0">
+    <comment ref="D121" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2906,14 +2975,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E118" authorId="0">
+    <comment ref="E121" authorId="0">
       <text>
         <r>
           <t>Destroy all creatures with no counters on them.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J118" authorId="0">
+    <comment ref="J121" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 3 generic
@@ -2921,7 +2990,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D119" authorId="0">
+    <comment ref="D122" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2931,14 +3000,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E119" authorId="0">
+    <comment ref="E122" authorId="0">
       <text>
         <r>
           <t>Target creature gets -4/-4 until end of turn. Proliferate. (Choose any number of permanents and/or players, then give each another counter of each kind already there.)</t>
         </r>
       </text>
     </comment>
-    <comment ref="J119" authorId="0">
+    <comment ref="J122" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 generic
@@ -2946,7 +3015,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D120" authorId="0">
+    <comment ref="D123" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2954,14 +3023,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E120" authorId="0">
+    <comment ref="E123" authorId="0">
       <text>
         <r>
           <t>Return any number of permanent cards with different names from your graveyard to the battlefield.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J120" authorId="0">
+    <comment ref="J123" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 2 white
@@ -2970,7 +3039,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D121" authorId="0">
+    <comment ref="D124" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -2978,14 +3047,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E121" authorId="0">
+    <comment ref="E124" authorId="0">
       <text>
         <r>
           <t>Exile target creature with mana value 3 or greater.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J121" authorId="0">
+    <comment ref="J124" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 1 generic
@@ -2993,7 +3062,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D122" authorId="0">
+    <comment ref="D125" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">Border: black
@@ -3003,14 +3072,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E122" authorId="0">
+    <comment ref="E125" authorId="0">
       <text>
         <r>
           <t>Converge — You draw X cards and lose X life, where X is the number of colors of mana spent to cast this spell.</t>
         </r>
       </text>
     </comment>
-    <comment ref="J122" authorId="0">
+    <comment ref="J125" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">➤ 2 generic
@@ -3023,7 +3092,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="735">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1615" uniqueCount="747">
   <si>
     <t>Commander (All) - All</t>
   </si>
@@ -4456,12 +4525,39 @@
     <t>Open Teleportation Circle</t>
   </si>
   <si>
+    <t>Abstruse Appropriation</t>
+  </si>
+  <si>
+    <t>Instant</t>
+  </si>
+  <si>
+    <t>177</t>
+  </si>
+  <si>
+    <t>0.22</t>
+  </si>
+  <si>
+    <t>Open Abstruse Appropriation</t>
+  </si>
+  <si>
+    <t>Abstruse Interference</t>
+  </si>
+  <si>
+    <t>ogw</t>
+  </si>
+  <si>
+    <t>Oath of the Gatewatch</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>Open Abstruse Interference</t>
+  </si>
+  <si>
     <t>Akroma's Will</t>
   </si>
   <si>
-    <t>Instant</t>
-  </si>
-  <si>
     <t>m3c</t>
   </si>
   <si>
@@ -4546,9 +4642,6 @@
     <t>Cyclonic Rift</t>
   </si>
   <si>
-    <t>40</t>
-  </si>
-  <si>
     <t>42.01</t>
   </si>
   <si>
@@ -4718,6 +4811,18 @@
   </si>
   <si>
     <t>Open Command Tower</t>
+  </si>
+  <si>
+    <t>Corrupted Crossroads</t>
+  </si>
+  <si>
+    <t>169</t>
+  </si>
+  <si>
+    <t>0.20</t>
+  </si>
+  <si>
+    <t>Open Corrupted Crossroads</t>
   </si>
   <si>
     <t>Dimir Guildgate</t>
@@ -5391,10 +5496,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5736,7 +5841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O322"/>
+  <dimension ref="A1:O325"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="49" customWidth="1"/>
@@ -9084,36 +9189,36 @@
         <v>19</v>
       </c>
       <c r="G72" s="15" t="s">
+        <v>403</v>
+      </c>
+      <c r="H72" s="15" t="s">
+        <v>404</v>
+      </c>
+      <c r="I72" s="15" t="s">
         <v>479</v>
       </c>
-      <c r="H72" s="15" t="s">
-        <v>480</v>
-      </c>
-      <c r="I72" s="15" t="s">
-        <v>481</v>
-      </c>
       <c r="J72" s="15" t="s">
-        <v>70</v>
+        <v>331</v>
       </c>
       <c r="K72" s="15">
         <v>4</v>
       </c>
       <c r="L72" s="15" t="s">
-        <v>62</v>
+        <v>24</v>
       </c>
       <c r="M72" s="15" t="s">
-        <v>62</v>
+        <v>332</v>
       </c>
       <c r="N72" s="15" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="O72" s="15" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="73" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B73" s="7">
         <v>1</v>
@@ -9128,39 +9233,39 @@
         <v>478</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G73" s="7" t="s">
+        <v>483</v>
+      </c>
+      <c r="H73" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="I73" s="7" t="s">
         <v>485</v>
       </c>
-      <c r="H73" s="7" t="s">
-        <v>486</v>
-      </c>
-      <c r="I73" s="7" t="s">
-        <v>487</v>
-      </c>
       <c r="J73" s="7" t="s">
-        <v>488</v>
+        <v>42</v>
       </c>
       <c r="K73" s="7">
         <v>3</v>
       </c>
       <c r="L73" s="7" t="s">
-        <v>332</v>
+        <v>24</v>
       </c>
       <c r="M73" s="7" t="s">
-        <v>332</v>
+        <v>43</v>
       </c>
       <c r="N73" s="7" t="s">
-        <v>489</v>
+        <v>174</v>
       </c>
       <c r="O73" s="7" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
     </row>
     <row r="74" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="B74" s="11">
         <v>1</v>
@@ -9178,36 +9283,36 @@
         <v>19</v>
       </c>
       <c r="G74" s="11" t="s">
-        <v>421</v>
+        <v>488</v>
       </c>
       <c r="H74" s="11" t="s">
-        <v>422</v>
+        <v>489</v>
       </c>
       <c r="I74" s="11" t="s">
+        <v>490</v>
+      </c>
+      <c r="J74" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="K74" s="11">
+        <v>4</v>
+      </c>
+      <c r="L74" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="M74" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="N74" s="11" t="s">
+        <v>491</v>
+      </c>
+      <c r="O74" s="11" t="s">
         <v>492</v>
-      </c>
-      <c r="J74" s="11" t="s">
-        <v>493</v>
-      </c>
-      <c r="K74" s="11">
-        <v>2</v>
-      </c>
-      <c r="L74" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="M74" s="11" t="s">
-        <v>219</v>
-      </c>
-      <c r="N74" s="11" t="s">
-        <v>494</v>
-      </c>
-      <c r="O74" s="11" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="75" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="B75" s="7">
         <v>1</v>
@@ -9225,36 +9330,36 @@
         <v>19</v>
       </c>
       <c r="G75" s="7" t="s">
+        <v>494</v>
+      </c>
+      <c r="H75" s="7" t="s">
+        <v>495</v>
+      </c>
+      <c r="I75" s="7" t="s">
+        <v>496</v>
+      </c>
+      <c r="J75" s="7" t="s">
         <v>497</v>
       </c>
-      <c r="H75" s="7" t="s">
+      <c r="K75" s="7">
+        <v>3</v>
+      </c>
+      <c r="L75" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="M75" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="N75" s="7" t="s">
         <v>498</v>
       </c>
-      <c r="I75" s="7" t="s">
+      <c r="O75" s="7" t="s">
         <v>499</v>
-      </c>
-      <c r="J75" s="7" t="s">
-        <v>337</v>
-      </c>
-      <c r="K75" s="7">
-        <v>4</v>
-      </c>
-      <c r="L75" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="M75" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="N75" s="7" t="s">
-        <v>500</v>
-      </c>
-      <c r="O75" s="7" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="76" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="B76" s="11">
         <v>1</v>
@@ -9272,36 +9377,36 @@
         <v>19</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>39</v>
+        <v>421</v>
       </c>
       <c r="H76" s="11" t="s">
-        <v>40</v>
+        <v>422</v>
       </c>
       <c r="I76" s="11" t="s">
-        <v>324</v>
+        <v>501</v>
       </c>
       <c r="J76" s="11" t="s">
+        <v>502</v>
+      </c>
+      <c r="K76" s="11">
+        <v>2</v>
+      </c>
+      <c r="L76" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="M76" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="N76" s="11" t="s">
         <v>503</v>
       </c>
-      <c r="K76" s="11">
-        <v>1</v>
-      </c>
-      <c r="L76" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="M76" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="N76" s="11" t="s">
+      <c r="O76" s="11" t="s">
         <v>504</v>
-      </c>
-      <c r="O76" s="11" t="s">
-        <v>505</v>
       </c>
     </row>
     <row r="77" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B77" s="7">
         <v>1</v>
@@ -9316,39 +9421,39 @@
         <v>478</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>202</v>
+        <v>506</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>203</v>
+        <v>507</v>
       </c>
       <c r="I77" s="7" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="J77" s="7" t="s">
-        <v>410</v>
+        <v>337</v>
       </c>
       <c r="K77" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L77" s="7" t="s">
-        <v>43</v>
+        <v>219</v>
       </c>
       <c r="M77" s="7" t="s">
-        <v>43</v>
+        <v>219</v>
       </c>
       <c r="N77" s="7" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="O77" s="7" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="78" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B78" s="11">
         <v>1</v>
@@ -9366,19 +9471,19 @@
         <v>19</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>97</v>
+        <v>39</v>
       </c>
       <c r="H78" s="11" t="s">
-        <v>98</v>
+        <v>40</v>
       </c>
       <c r="I78" s="11" t="s">
-        <v>511</v>
+        <v>324</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>189</v>
+        <v>512</v>
       </c>
       <c r="K78" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L78" s="11" t="s">
         <v>34</v>
@@ -9387,15 +9492,15 @@
         <v>34</v>
       </c>
       <c r="N78" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="O78" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
     </row>
     <row r="79" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B79" s="7">
         <v>1</v>
@@ -9410,39 +9515,39 @@
         <v>478</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>136</v>
+        <v>49</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>30</v>
+        <v>202</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>31</v>
+        <v>203</v>
       </c>
       <c r="I79" s="7" t="s">
-        <v>515</v>
+        <v>485</v>
       </c>
       <c r="J79" s="7" t="s">
-        <v>516</v>
+        <v>410</v>
       </c>
       <c r="K79" s="7">
         <v>2</v>
       </c>
       <c r="L79" s="7" t="s">
-        <v>291</v>
+        <v>43</v>
       </c>
       <c r="M79" s="7" t="s">
-        <v>291</v>
+        <v>43</v>
       </c>
       <c r="N79" s="7" t="s">
+        <v>516</v>
+      </c>
+      <c r="O79" s="7" t="s">
         <v>517</v>
-      </c>
-      <c r="O79" s="7" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="80" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="10" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B80" s="11">
         <v>1</v>
@@ -9457,39 +9562,39 @@
         <v>478</v>
       </c>
       <c r="F80" s="11" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="G80" s="11" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="H80" s="11" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="I80" s="11" t="s">
+        <v>519</v>
+      </c>
+      <c r="J80" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="K80" s="11">
+        <v>4</v>
+      </c>
+      <c r="L80" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="M80" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="N80" s="11" t="s">
         <v>520</v>
       </c>
-      <c r="J80" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="K80" s="11">
-        <v>1</v>
-      </c>
-      <c r="L80" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="M80" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="N80" s="11" t="s">
+      <c r="O80" s="11" t="s">
         <v>521</v>
-      </c>
-      <c r="O80" s="11" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="81" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B81" s="7">
         <v>1</v>
@@ -9504,39 +9609,39 @@
         <v>478</v>
       </c>
       <c r="F81" s="7" t="s">
-        <v>19</v>
+        <v>136</v>
       </c>
       <c r="G81" s="7" t="s">
-        <v>97</v>
+        <v>30</v>
       </c>
       <c r="H81" s="7" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="I81" s="7" t="s">
-        <v>499</v>
+        <v>523</v>
       </c>
       <c r="J81" s="7" t="s">
-        <v>42</v>
+        <v>524</v>
       </c>
       <c r="K81" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L81" s="7" t="s">
-        <v>43</v>
+        <v>291</v>
       </c>
       <c r="M81" s="7" t="s">
-        <v>43</v>
+        <v>291</v>
       </c>
       <c r="N81" s="7" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="O81" s="7" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="82" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B82" s="11">
         <v>1</v>
@@ -9551,39 +9656,39 @@
         <v>478</v>
       </c>
       <c r="F82" s="11" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G82" s="11" t="s">
-        <v>527</v>
+        <v>76</v>
       </c>
       <c r="H82" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="I82" s="11" t="s">
         <v>528</v>
       </c>
-      <c r="I82" s="11" t="s">
-        <v>41</v>
-      </c>
       <c r="J82" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="K82" s="11">
+        <v>1</v>
+      </c>
+      <c r="L82" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="M82" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="N82" s="11" t="s">
         <v>529</v>
       </c>
-      <c r="K82" s="11">
-        <v>3</v>
-      </c>
-      <c r="L82" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="M82" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="N82" s="11" t="s">
+      <c r="O82" s="11" t="s">
         <v>530</v>
-      </c>
-      <c r="O82" s="11" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="83" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B83" s="7">
         <v>1</v>
@@ -9598,227 +9703,227 @@
         <v>478</v>
       </c>
       <c r="F83" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G83" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H83" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="I83" s="7" t="s">
+        <v>508</v>
+      </c>
+      <c r="J83" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K83" s="7">
+        <v>3</v>
+      </c>
+      <c r="L83" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="M83" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="N83" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="O83" s="7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="10" t="s">
+        <v>534</v>
+      </c>
+      <c r="B84" s="11">
+        <v>1</v>
+      </c>
+      <c r="C84" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D84" s="11" t="s">
+        <v>478</v>
+      </c>
+      <c r="E84" s="11" t="s">
+        <v>478</v>
+      </c>
+      <c r="F84" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G84" s="11" t="s">
+        <v>535</v>
+      </c>
+      <c r="H84" s="11" t="s">
+        <v>536</v>
+      </c>
+      <c r="I84" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="J84" s="11" t="s">
+        <v>537</v>
+      </c>
+      <c r="K84" s="11">
+        <v>3</v>
+      </c>
+      <c r="L84" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M84" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="N84" s="11" t="s">
+        <v>538</v>
+      </c>
+      <c r="O84" s="11" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="B85" s="7">
+        <v>1</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="F85" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G83" s="7" t="s">
-        <v>533</v>
-      </c>
-      <c r="H83" s="7" t="s">
-        <v>534</v>
-      </c>
-      <c r="I83" s="7" t="s">
-        <v>535</v>
-      </c>
-      <c r="J83" s="7" t="s">
-        <v>536</v>
-      </c>
-      <c r="K83" s="7">
+      <c r="G85" s="7" t="s">
+        <v>541</v>
+      </c>
+      <c r="H85" s="7" t="s">
+        <v>542</v>
+      </c>
+      <c r="I85" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="J85" s="7" t="s">
+        <v>544</v>
+      </c>
+      <c r="K85" s="7">
         <v>1</v>
       </c>
-      <c r="L83" s="7" t="s">
+      <c r="L85" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="M83" s="7" t="s">
+      <c r="M85" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="N83" s="7" t="s">
-        <v>537</v>
-      </c>
-      <c r="O83" s="7" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="84" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="14" t="s">
-        <v>539</v>
-      </c>
-      <c r="B84" s="15">
+      <c r="N85" s="7" t="s">
+        <v>545</v>
+      </c>
+      <c r="O85" s="7" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="14" t="s">
+        <v>547</v>
+      </c>
+      <c r="B86" s="15">
         <v>1</v>
       </c>
-      <c r="C84" s="15" t="s">
+      <c r="C86" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D84" s="15" t="s">
-        <v>540</v>
-      </c>
-      <c r="E84" s="15" t="s">
-        <v>540</v>
-      </c>
-      <c r="F84" s="15" t="s">
+      <c r="D86" s="15" t="s">
+        <v>548</v>
+      </c>
+      <c r="E86" s="15" t="s">
+        <v>548</v>
+      </c>
+      <c r="F86" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="G84" s="15" t="s">
-        <v>541</v>
-      </c>
-      <c r="H84" s="15" t="s">
-        <v>542</v>
-      </c>
-      <c r="I84" s="15" t="s">
-        <v>543</v>
-      </c>
-      <c r="J84" s="15" t="s">
+      <c r="G86" s="15" t="s">
+        <v>549</v>
+      </c>
+      <c r="H86" s="15" t="s">
+        <v>550</v>
+      </c>
+      <c r="I86" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="J86" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="K84" s="15">
+      <c r="K86" s="15">
         <v>0</v>
       </c>
-      <c r="L84" s="15" t="s">
+      <c r="L86" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="M84" s="15" t="s">
+      <c r="M86" s="15" t="s">
         <v>437</v>
       </c>
-      <c r="N84" s="15" t="s">
-        <v>544</v>
-      </c>
-      <c r="O84" s="15" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="85" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="8" t="s">
-        <v>539</v>
-      </c>
-      <c r="B85" s="9">
+      <c r="N86" s="15" t="s">
+        <v>552</v>
+      </c>
+      <c r="O86" s="15" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="87" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="B87" s="9">
         <v>1</v>
       </c>
-      <c r="C85" s="9" t="s">
+      <c r="C87" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D85" s="9" t="s">
-        <v>540</v>
-      </c>
-      <c r="E85" s="9" t="s">
-        <v>540</v>
-      </c>
-      <c r="F85" s="9" t="s">
+      <c r="D87" s="9" t="s">
+        <v>548</v>
+      </c>
+      <c r="E87" s="9" t="s">
+        <v>548</v>
+      </c>
+      <c r="F87" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="G85" s="9" t="s">
-        <v>541</v>
-      </c>
-      <c r="H85" s="9" t="s">
-        <v>542</v>
-      </c>
-      <c r="I85" s="9" t="s">
-        <v>543</v>
-      </c>
-      <c r="J85" s="9" t="s">
+      <c r="G87" s="9" t="s">
+        <v>549</v>
+      </c>
+      <c r="H87" s="9" t="s">
+        <v>550</v>
+      </c>
+      <c r="I87" s="9" t="s">
+        <v>551</v>
+      </c>
+      <c r="J87" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="K85" s="9">
+      <c r="K87" s="9">
         <v>0</v>
       </c>
-      <c r="L85" s="9" t="s">
+      <c r="L87" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="M85" s="9" t="s">
+      <c r="M87" s="9" t="s">
         <v>437</v>
       </c>
-      <c r="N85" s="9" t="s">
-        <v>544</v>
-      </c>
-      <c r="O85" s="9" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="86" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="10" t="s">
-        <v>546</v>
-      </c>
-      <c r="B86" s="11">
-        <v>1</v>
-      </c>
-      <c r="C86" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D86" s="11" t="s">
-        <v>540</v>
-      </c>
-      <c r="E86" s="11" t="s">
-        <v>540</v>
-      </c>
-      <c r="F86" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G86" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="H86" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="I86" s="11" t="s">
-        <v>547</v>
-      </c>
-      <c r="J86" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="K86" s="11">
-        <v>0</v>
-      </c>
-      <c r="L86" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="M86" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="N86" s="11" t="s">
-        <v>548</v>
-      </c>
-      <c r="O86" s="11" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="87" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="6" t="s">
-        <v>550</v>
-      </c>
-      <c r="B87" s="7">
-        <v>1</v>
-      </c>
-      <c r="C87" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D87" s="7" t="s">
-        <v>540</v>
-      </c>
-      <c r="E87" s="7" t="s">
-        <v>551</v>
-      </c>
-      <c r="F87" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="G87" s="7" t="s">
+      <c r="N87" s="9" t="s">
         <v>552</v>
       </c>
-      <c r="H87" s="7" t="s">
+      <c r="O87" s="9" t="s">
         <v>553</v>
-      </c>
-      <c r="I87" s="7" t="s">
-        <v>554</v>
-      </c>
-      <c r="J87" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="K87" s="7">
-        <v>0</v>
-      </c>
-      <c r="L87" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="M87" s="7" t="s">
-        <v>437</v>
-      </c>
-      <c r="N87" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="O87" s="7" t="s">
-        <v>555</v>
       </c>
     </row>
     <row r="88" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="10" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="B88" s="11">
         <v>1</v>
@@ -9827,22 +9932,22 @@
         <v>17</v>
       </c>
       <c r="D88" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E88" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="F88" s="11" t="s">
         <v>19</v>
       </c>
       <c r="G88" s="11" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="H88" s="11" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="I88" s="11" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="J88" s="11" t="s">
         <v>24</v>
@@ -9854,18 +9959,18 @@
         <v>24</v>
       </c>
       <c r="M88" s="11" t="s">
-        <v>558</v>
+        <v>114</v>
       </c>
       <c r="N88" s="11" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="O88" s="11" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
     </row>
     <row r="89" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="B89" s="7">
         <v>1</v>
@@ -9874,22 +9979,22 @@
         <v>17</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E89" s="7" t="s">
-        <v>540</v>
+        <v>559</v>
       </c>
       <c r="F89" s="7" t="s">
         <v>38</v>
       </c>
       <c r="G89" s="7" t="s">
+        <v>560</v>
+      </c>
+      <c r="H89" s="7" t="s">
+        <v>561</v>
+      </c>
+      <c r="I89" s="7" t="s">
         <v>562</v>
-      </c>
-      <c r="H89" s="7" t="s">
-        <v>563</v>
-      </c>
-      <c r="I89" s="7" t="s">
-        <v>547</v>
       </c>
       <c r="J89" s="7" t="s">
         <v>24</v>
@@ -9901,18 +10006,18 @@
         <v>24</v>
       </c>
       <c r="M89" s="7" t="s">
-        <v>24</v>
+        <v>437</v>
       </c>
       <c r="N89" s="7" t="s">
-        <v>355</v>
+        <v>190</v>
       </c>
       <c r="O89" s="7" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="90" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="10" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B90" s="11">
         <v>1</v>
@@ -9921,22 +10026,22 @@
         <v>17</v>
       </c>
       <c r="D90" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E90" s="11" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="F90" s="11" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="G90" s="11" t="s">
-        <v>277</v>
+        <v>30</v>
       </c>
       <c r="H90" s="11" t="s">
-        <v>278</v>
+        <v>31</v>
       </c>
       <c r="I90" s="11" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="J90" s="11" t="s">
         <v>24</v>
@@ -9948,18 +10053,18 @@
         <v>24</v>
       </c>
       <c r="M90" s="11" t="s">
-        <v>291</v>
+        <v>566</v>
       </c>
       <c r="N90" s="11" t="s">
-        <v>140</v>
+        <v>567</v>
       </c>
       <c r="O90" s="11" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="91" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B91" s="7">
         <v>1</v>
@@ -9968,22 +10073,22 @@
         <v>17</v>
       </c>
       <c r="D91" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E91" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="F91" s="7" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G91" s="7" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="H91" s="7" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="I91" s="7" t="s">
-        <v>571</v>
+        <v>555</v>
       </c>
       <c r="J91" s="7" t="s">
         <v>24</v>
@@ -9995,18 +10100,18 @@
         <v>24</v>
       </c>
       <c r="M91" s="7" t="s">
-        <v>437</v>
+        <v>24</v>
       </c>
       <c r="N91" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="O91" s="7" t="s">
         <v>572</v>
-      </c>
-      <c r="O91" s="7" t="s">
-        <v>573</v>
       </c>
     </row>
     <row r="92" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B92" s="11">
         <v>1</v>
@@ -10015,22 +10120,22 @@
         <v>17</v>
       </c>
       <c r="D92" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E92" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="F92" s="11" t="s">
         <v>19</v>
       </c>
       <c r="G92" s="11" t="s">
-        <v>575</v>
+        <v>483</v>
       </c>
       <c r="H92" s="11" t="s">
-        <v>576</v>
+        <v>484</v>
       </c>
       <c r="I92" s="11" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="J92" s="11" t="s">
         <v>24</v>
@@ -10045,15 +10150,15 @@
         <v>24</v>
       </c>
       <c r="N92" s="11" t="s">
-        <v>504</v>
+        <v>575</v>
       </c>
       <c r="O92" s="11" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="93" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B93" s="7">
         <v>1</v>
@@ -10062,22 +10167,22 @@
         <v>17</v>
       </c>
       <c r="D93" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E93" s="7" t="s">
-        <v>580</v>
+        <v>559</v>
       </c>
       <c r="F93" s="7" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G93" s="7" t="s">
-        <v>118</v>
+        <v>277</v>
       </c>
       <c r="H93" s="7" t="s">
-        <v>119</v>
+        <v>278</v>
       </c>
       <c r="I93" s="7" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="J93" s="7" t="s">
         <v>24</v>
@@ -10089,18 +10194,18 @@
         <v>24</v>
       </c>
       <c r="M93" s="7" t="s">
-        <v>582</v>
+        <v>291</v>
       </c>
       <c r="N93" s="7" t="s">
-        <v>583</v>
+        <v>140</v>
       </c>
       <c r="O93" s="7" t="s">
-        <v>584</v>
+        <v>579</v>
       </c>
     </row>
     <row r="94" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="10" t="s">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="B94" s="11">
         <v>1</v>
@@ -10109,22 +10214,22 @@
         <v>17</v>
       </c>
       <c r="D94" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E94" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="F94" s="11" t="s">
         <v>19</v>
       </c>
       <c r="G94" s="11" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="H94" s="11" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="I94" s="11" t="s">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="J94" s="11" t="s">
         <v>24</v>
@@ -10136,18 +10241,18 @@
         <v>24</v>
       </c>
       <c r="M94" s="11" t="s">
-        <v>24</v>
+        <v>437</v>
       </c>
       <c r="N94" s="11" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="O94" s="11" t="s">
-        <v>590</v>
+        <v>585</v>
       </c>
     </row>
     <row r="95" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
-        <v>591</v>
+        <v>586</v>
       </c>
       <c r="B95" s="7">
         <v>1</v>
@@ -10156,22 +10261,22 @@
         <v>17</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="F95" s="7" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="G95" s="7" t="s">
-        <v>97</v>
+        <v>587</v>
       </c>
       <c r="H95" s="7" t="s">
-        <v>98</v>
+        <v>588</v>
       </c>
       <c r="I95" s="7" t="s">
-        <v>204</v>
+        <v>589</v>
       </c>
       <c r="J95" s="7" t="s">
         <v>24</v>
@@ -10186,15 +10291,15 @@
         <v>24</v>
       </c>
       <c r="N95" s="7" t="s">
-        <v>338</v>
+        <v>513</v>
       </c>
       <c r="O95" s="7" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="96" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="10" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B96" s="11">
         <v>1</v>
@@ -10203,22 +10308,22 @@
         <v>17</v>
       </c>
       <c r="D96" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E96" s="11" t="s">
-        <v>540</v>
+        <v>592</v>
       </c>
       <c r="F96" s="11" t="s">
         <v>19</v>
       </c>
       <c r="G96" s="11" t="s">
-        <v>76</v>
+        <v>118</v>
       </c>
       <c r="H96" s="11" t="s">
-        <v>77</v>
+        <v>119</v>
       </c>
       <c r="I96" s="11" t="s">
-        <v>554</v>
+        <v>593</v>
       </c>
       <c r="J96" s="11" t="s">
         <v>24</v>
@@ -10230,18 +10335,18 @@
         <v>24</v>
       </c>
       <c r="M96" s="11" t="s">
-        <v>24</v>
+        <v>594</v>
       </c>
       <c r="N96" s="11" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="O96" s="11" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
     </row>
     <row r="97" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B97" s="7">
         <v>1</v>
@@ -10250,22 +10355,22 @@
         <v>17</v>
       </c>
       <c r="D97" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E97" s="7" t="s">
-        <v>597</v>
+        <v>548</v>
       </c>
       <c r="F97" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G97" s="7" t="s">
-        <v>164</v>
+        <v>598</v>
       </c>
       <c r="H97" s="7" t="s">
-        <v>165</v>
+        <v>599</v>
       </c>
       <c r="I97" s="7" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="J97" s="7" t="s">
         <v>24</v>
@@ -10277,18 +10382,18 @@
         <v>24</v>
       </c>
       <c r="M97" s="7" t="s">
-        <v>599</v>
+        <v>24</v>
       </c>
       <c r="N97" s="7" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="O97" s="7" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="98" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="10" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B98" s="11">
         <v>1</v>
@@ -10297,22 +10402,22 @@
         <v>17</v>
       </c>
       <c r="D98" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E98" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="F98" s="11" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G98" s="11" t="s">
-        <v>603</v>
+        <v>97</v>
       </c>
       <c r="H98" s="11" t="s">
-        <v>604</v>
+        <v>98</v>
       </c>
       <c r="I98" s="11" t="s">
-        <v>324</v>
+        <v>204</v>
       </c>
       <c r="J98" s="11" t="s">
         <v>24</v>
@@ -10324,18 +10429,18 @@
         <v>24</v>
       </c>
       <c r="M98" s="11" t="s">
-        <v>437</v>
+        <v>24</v>
       </c>
       <c r="N98" s="11" t="s">
-        <v>605</v>
+        <v>338</v>
       </c>
       <c r="O98" s="11" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="99" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B99" s="7">
         <v>1</v>
@@ -10344,22 +10449,22 @@
         <v>17</v>
       </c>
       <c r="D99" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E99" s="7" t="s">
-        <v>608</v>
+        <v>548</v>
       </c>
       <c r="F99" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G99" s="7" t="s">
-        <v>164</v>
+        <v>76</v>
       </c>
       <c r="H99" s="7" t="s">
-        <v>165</v>
+        <v>77</v>
       </c>
       <c r="I99" s="7" t="s">
-        <v>609</v>
+        <v>562</v>
       </c>
       <c r="J99" s="7" t="s">
         <v>24</v>
@@ -10371,18 +10476,18 @@
         <v>24</v>
       </c>
       <c r="M99" s="7" t="s">
-        <v>610</v>
+        <v>24</v>
       </c>
       <c r="N99" s="7" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="O99" s="7" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
     </row>
     <row r="100" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="10" t="s">
-        <v>613</v>
+        <v>608</v>
       </c>
       <c r="B100" s="11">
         <v>1</v>
@@ -10391,22 +10496,22 @@
         <v>17</v>
       </c>
       <c r="D100" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E100" s="11" t="s">
-        <v>540</v>
+        <v>609</v>
       </c>
       <c r="F100" s="11" t="s">
         <v>19</v>
       </c>
       <c r="G100" s="11" t="s">
-        <v>614</v>
+        <v>164</v>
       </c>
       <c r="H100" s="11" t="s">
-        <v>615</v>
+        <v>165</v>
       </c>
       <c r="I100" s="11" t="s">
-        <v>616</v>
+        <v>610</v>
       </c>
       <c r="J100" s="11" t="s">
         <v>24</v>
@@ -10418,18 +10523,18 @@
         <v>24</v>
       </c>
       <c r="M100" s="11" t="s">
-        <v>332</v>
+        <v>611</v>
       </c>
       <c r="N100" s="11" t="s">
-        <v>617</v>
+        <v>612</v>
       </c>
       <c r="O100" s="11" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
     </row>
     <row r="101" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
-        <v>619</v>
+        <v>614</v>
       </c>
       <c r="B101" s="7">
         <v>1</v>
@@ -10438,22 +10543,22 @@
         <v>17</v>
       </c>
       <c r="D101" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>620</v>
+        <v>548</v>
       </c>
       <c r="F101" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G101" s="7" t="s">
-        <v>421</v>
+        <v>615</v>
       </c>
       <c r="H101" s="7" t="s">
-        <v>422</v>
+        <v>616</v>
       </c>
       <c r="I101" s="7" t="s">
-        <v>621</v>
+        <v>324</v>
       </c>
       <c r="J101" s="7" t="s">
         <v>24</v>
@@ -10465,18 +10570,18 @@
         <v>24</v>
       </c>
       <c r="M101" s="7" t="s">
-        <v>291</v>
+        <v>437</v>
       </c>
       <c r="N101" s="7" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="O101" s="7" t="s">
-        <v>623</v>
+        <v>618</v>
       </c>
     </row>
     <row r="102" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="10" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="B102" s="11">
         <v>1</v>
@@ -10485,22 +10590,22 @@
         <v>17</v>
       </c>
       <c r="D102" s="11" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E102" s="11" t="s">
-        <v>540</v>
+        <v>620</v>
       </c>
       <c r="F102" s="11" t="s">
         <v>19</v>
       </c>
       <c r="G102" s="11" t="s">
-        <v>97</v>
+        <v>164</v>
       </c>
       <c r="H102" s="11" t="s">
-        <v>98</v>
+        <v>165</v>
       </c>
       <c r="I102" s="11" t="s">
-        <v>625</v>
+        <v>621</v>
       </c>
       <c r="J102" s="11" t="s">
         <v>24</v>
@@ -10512,18 +10617,18 @@
         <v>24</v>
       </c>
       <c r="M102" s="11" t="s">
-        <v>332</v>
+        <v>622</v>
       </c>
       <c r="N102" s="11" t="s">
-        <v>430</v>
+        <v>623</v>
       </c>
       <c r="O102" s="11" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="103" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="B103" s="7">
         <v>1</v>
@@ -10532,22 +10637,22 @@
         <v>17</v>
       </c>
       <c r="D103" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E103" s="7" t="s">
-        <v>628</v>
+        <v>548</v>
       </c>
       <c r="F103" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G103" s="7" t="s">
-        <v>118</v>
+        <v>626</v>
       </c>
       <c r="H103" s="7" t="s">
-        <v>119</v>
+        <v>627</v>
       </c>
       <c r="I103" s="7" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="J103" s="7" t="s">
         <v>24</v>
@@ -10559,65 +10664,65 @@
         <v>24</v>
       </c>
       <c r="M103" s="7" t="s">
-        <v>366</v>
+        <v>332</v>
       </c>
       <c r="N103" s="7" t="s">
+        <v>629</v>
+      </c>
+      <c r="O103" s="7" t="s">
         <v>630</v>
       </c>
-      <c r="O103" s="7" t="s">
+    </row>
+    <row r="104" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A104" s="10" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="104" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="14" t="s">
+      <c r="B104" s="11">
+        <v>1</v>
+      </c>
+      <c r="C104" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D104" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="E104" s="11" t="s">
         <v>632</v>
       </c>
-      <c r="B104" s="15">
-        <v>1</v>
-      </c>
-      <c r="C104" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D104" s="15" t="s">
+      <c r="F104" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G104" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="H104" s="11" t="s">
+        <v>422</v>
+      </c>
+      <c r="I104" s="11" t="s">
         <v>633</v>
       </c>
-      <c r="E104" s="15" t="s">
+      <c r="J104" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K104" s="11">
+        <v>0</v>
+      </c>
+      <c r="L104" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="M104" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="N104" s="11" t="s">
         <v>634</v>
       </c>
-      <c r="F104" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="G104" s="15" t="s">
-        <v>533</v>
-      </c>
-      <c r="H104" s="15" t="s">
-        <v>534</v>
-      </c>
-      <c r="I104" s="15" t="s">
+      <c r="O104" s="11" t="s">
         <v>635</v>
-      </c>
-      <c r="J104" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="K104" s="15">
-        <v>0</v>
-      </c>
-      <c r="L104" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="M104" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="N104" s="15" t="s">
-        <v>636</v>
-      </c>
-      <c r="O104" s="15" t="s">
-        <v>637</v>
       </c>
     </row>
     <row r="105" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="B105" s="7">
         <v>1</v>
@@ -10626,22 +10731,22 @@
         <v>17</v>
       </c>
       <c r="D105" s="7" t="s">
-        <v>633</v>
+        <v>548</v>
       </c>
       <c r="E105" s="7" t="s">
-        <v>634</v>
+        <v>548</v>
       </c>
       <c r="F105" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G105" s="7" t="s">
-        <v>533</v>
+        <v>97</v>
       </c>
       <c r="H105" s="7" t="s">
-        <v>534</v>
+        <v>98</v>
       </c>
       <c r="I105" s="7" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="J105" s="7" t="s">
         <v>24</v>
@@ -10653,18 +10758,18 @@
         <v>24</v>
       </c>
       <c r="M105" s="7" t="s">
-        <v>62</v>
+        <v>332</v>
       </c>
       <c r="N105" s="7" t="s">
-        <v>640</v>
+        <v>430</v>
       </c>
       <c r="O105" s="7" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
     </row>
     <row r="106" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="B106" s="11">
         <v>1</v>
@@ -10673,22 +10778,22 @@
         <v>17</v>
       </c>
       <c r="D106" s="11" t="s">
-        <v>633</v>
+        <v>548</v>
       </c>
       <c r="E106" s="11" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="F106" s="11" t="s">
         <v>19</v>
       </c>
       <c r="G106" s="11" t="s">
-        <v>58</v>
+        <v>118</v>
       </c>
       <c r="H106" s="11" t="s">
-        <v>59</v>
+        <v>119</v>
       </c>
       <c r="I106" s="11" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="J106" s="11" t="s">
         <v>24</v>
@@ -10700,18 +10805,18 @@
         <v>24</v>
       </c>
       <c r="M106" s="11" t="s">
-        <v>24</v>
+        <v>366</v>
       </c>
       <c r="N106" s="11" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="O106" s="11" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="107" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="12" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="B107" s="13">
         <v>1</v>
@@ -10720,22 +10825,22 @@
         <v>17</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="E107" s="13" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="F107" s="13" t="s">
         <v>19</v>
       </c>
       <c r="G107" s="13" t="s">
-        <v>245</v>
+        <v>541</v>
       </c>
       <c r="H107" s="13" t="s">
-        <v>246</v>
+        <v>542</v>
       </c>
       <c r="I107" s="13" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="J107" s="13" t="s">
         <v>24</v>
@@ -10747,253 +10852,253 @@
         <v>24</v>
       </c>
       <c r="M107" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="N107" s="13" t="s">
+        <v>648</v>
+      </c>
+      <c r="O107" s="13" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="108" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A108" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="B108" s="11">
+        <v>1</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D108" s="11" t="s">
+        <v>645</v>
+      </c>
+      <c r="E108" s="11" t="s">
+        <v>646</v>
+      </c>
+      <c r="F108" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G108" s="11" t="s">
+        <v>541</v>
+      </c>
+      <c r="H108" s="11" t="s">
+        <v>542</v>
+      </c>
+      <c r="I108" s="11" t="s">
+        <v>651</v>
+      </c>
+      <c r="J108" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="N107" s="13" t="s">
-        <v>650</v>
-      </c>
-      <c r="O107" s="13" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="108" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="14" t="s">
+      <c r="K108" s="11">
+        <v>0</v>
+      </c>
+      <c r="L108" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="M108" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="N108" s="11" t="s">
         <v>652</v>
       </c>
-      <c r="B108" s="15">
+      <c r="O108" s="11" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="109" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="B109" s="7">
         <v>1</v>
       </c>
-      <c r="C108" s="15" t="s">
+      <c r="C109" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D108" s="15" t="s">
-        <v>653</v>
-      </c>
-      <c r="E108" s="15" t="s">
-        <v>654</v>
-      </c>
-      <c r="F108" s="15" t="s">
+      <c r="D109" s="7" t="s">
+        <v>645</v>
+      </c>
+      <c r="E109" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="F109" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G109" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="H109" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="I109" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="J109" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K109" s="7">
+        <v>0</v>
+      </c>
+      <c r="L109" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M109" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N109" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="O109" s="7" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="110" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A110" s="14" t="s">
+        <v>658</v>
+      </c>
+      <c r="B110" s="15">
+        <v>1</v>
+      </c>
+      <c r="C110" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D110" s="15" t="s">
+        <v>659</v>
+      </c>
+      <c r="E110" s="15" t="s">
+        <v>660</v>
+      </c>
+      <c r="F110" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G110" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="H110" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="I110" s="15" t="s">
+        <v>661</v>
+      </c>
+      <c r="J110" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="K110" s="15">
+        <v>0</v>
+      </c>
+      <c r="L110" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="M110" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="N110" s="15" t="s">
+        <v>662</v>
+      </c>
+      <c r="O110" s="15" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="111" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A111" s="12" t="s">
+        <v>664</v>
+      </c>
+      <c r="B111" s="13">
+        <v>1</v>
+      </c>
+      <c r="C111" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D111" s="13" t="s">
+        <v>665</v>
+      </c>
+      <c r="E111" s="13" t="s">
+        <v>666</v>
+      </c>
+      <c r="F111" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="G108" s="15" t="s">
+      <c r="G111" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="H108" s="15" t="s">
+      <c r="H111" s="13" t="s">
         <v>380</v>
       </c>
-      <c r="I108" s="15" t="s">
-        <v>581</v>
-      </c>
-      <c r="J108" s="15" t="s">
+      <c r="I111" s="13" t="s">
+        <v>593</v>
+      </c>
+      <c r="J111" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="K108" s="15">
+      <c r="K111" s="13">
         <v>0</v>
       </c>
-      <c r="L108" s="15" t="s">
+      <c r="L111" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="M108" s="15" t="s">
-        <v>655</v>
-      </c>
-      <c r="N108" s="15" t="s">
-        <v>656</v>
-      </c>
-      <c r="O108" s="15" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="109" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="12" t="s">
-        <v>658</v>
-      </c>
-      <c r="B109" s="13">
+      <c r="M111" s="13" t="s">
+        <v>667</v>
+      </c>
+      <c r="N111" s="13" t="s">
+        <v>668</v>
+      </c>
+      <c r="O111" s="13" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="112" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A112" s="14" t="s">
+        <v>670</v>
+      </c>
+      <c r="B112" s="15">
         <v>1</v>
       </c>
-      <c r="C109" s="13" t="s">
+      <c r="C112" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D109" s="13" t="s">
-        <v>659</v>
-      </c>
-      <c r="E109" s="13" t="s">
-        <v>660</v>
-      </c>
-      <c r="F109" s="13" t="s">
+      <c r="D112" s="15" t="s">
+        <v>671</v>
+      </c>
+      <c r="E112" s="15" t="s">
+        <v>672</v>
+      </c>
+      <c r="F112" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G109" s="13" t="s">
+      <c r="G112" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="H109" s="13" t="s">
+      <c r="H112" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="I109" s="13" t="s">
-        <v>661</v>
-      </c>
-      <c r="J109" s="13" t="s">
-        <v>662</v>
-      </c>
-      <c r="K109" s="13">
+      <c r="I112" s="15" t="s">
+        <v>673</v>
+      </c>
+      <c r="J112" s="15" t="s">
+        <v>674</v>
+      </c>
+      <c r="K112" s="15">
         <v>4</v>
       </c>
-      <c r="L109" s="13" t="s">
-        <v>558</v>
-      </c>
-      <c r="M109" s="13" t="s">
-        <v>558</v>
-      </c>
-      <c r="N109" s="13" t="s">
-        <v>663</v>
-      </c>
-      <c r="O109" s="13" t="s">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="110" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="10" t="s">
-        <v>665</v>
-      </c>
-      <c r="B110" s="11">
-        <v>1</v>
-      </c>
-      <c r="C110" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D110" s="11" t="s">
-        <v>659</v>
-      </c>
-      <c r="E110" s="11" t="s">
-        <v>666</v>
-      </c>
-      <c r="F110" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G110" s="11" t="s">
-        <v>527</v>
-      </c>
-      <c r="H110" s="11" t="s">
-        <v>528</v>
-      </c>
-      <c r="I110" s="11" t="s">
-        <v>667</v>
-      </c>
-      <c r="J110" s="11" t="s">
-        <v>668</v>
-      </c>
-      <c r="K110" s="11">
-        <v>3</v>
-      </c>
-      <c r="L110" s="11" t="s">
-        <v>599</v>
-      </c>
-      <c r="M110" s="11" t="s">
-        <v>599</v>
-      </c>
-      <c r="N110" s="11" t="s">
-        <v>669</v>
-      </c>
-      <c r="O110" s="11" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="111" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="6" t="s">
-        <v>671</v>
-      </c>
-      <c r="B111" s="7">
-        <v>1</v>
-      </c>
-      <c r="C111" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D111" s="7" t="s">
-        <v>659</v>
-      </c>
-      <c r="E111" s="7" t="s">
-        <v>672</v>
-      </c>
-      <c r="F111" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="G111" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="H111" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="I111" s="7" t="s">
-        <v>673</v>
-      </c>
-      <c r="J111" s="7" t="s">
-        <v>674</v>
-      </c>
-      <c r="K111" s="7">
-        <v>3</v>
-      </c>
-      <c r="L111" s="7" t="s">
-        <v>291</v>
-      </c>
-      <c r="M111" s="7" t="s">
-        <v>291</v>
-      </c>
-      <c r="N111" s="7" t="s">
+      <c r="L112" s="15" t="s">
+        <v>566</v>
+      </c>
+      <c r="M112" s="15" t="s">
+        <v>566</v>
+      </c>
+      <c r="N112" s="15" t="s">
         <v>675</v>
       </c>
-      <c r="O111" s="7" t="s">
+      <c r="O112" s="15" t="s">
         <v>676</v>
-      </c>
-    </row>
-    <row r="112" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="10" t="s">
-        <v>677</v>
-      </c>
-      <c r="B112" s="11">
-        <v>1</v>
-      </c>
-      <c r="C112" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D112" s="11" t="s">
-        <v>659</v>
-      </c>
-      <c r="E112" s="11" t="s">
-        <v>678</v>
-      </c>
-      <c r="F112" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G112" s="11" t="s">
-        <v>303</v>
-      </c>
-      <c r="H112" s="11" t="s">
-        <v>304</v>
-      </c>
-      <c r="I112" s="11" t="s">
-        <v>679</v>
-      </c>
-      <c r="J112" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="K112" s="11">
-        <v>4</v>
-      </c>
-      <c r="L112" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="M112" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="N112" s="11" t="s">
-        <v>680</v>
-      </c>
-      <c r="O112" s="11" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="113" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="6" t="s">
-        <v>682</v>
+        <v>677</v>
       </c>
       <c r="B113" s="7">
         <v>1</v>
@@ -11002,45 +11107,45 @@
         <v>17</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>659</v>
+        <v>671</v>
       </c>
       <c r="E113" s="7" t="s">
-        <v>683</v>
+        <v>678</v>
       </c>
       <c r="F113" s="7" t="s">
-        <v>136</v>
+        <v>49</v>
       </c>
       <c r="G113" s="7" t="s">
-        <v>303</v>
+        <v>535</v>
       </c>
       <c r="H113" s="7" t="s">
-        <v>304</v>
+        <v>536</v>
       </c>
       <c r="I113" s="7" t="s">
-        <v>684</v>
+        <v>679</v>
       </c>
       <c r="J113" s="7" t="s">
-        <v>529</v>
+        <v>680</v>
       </c>
       <c r="K113" s="7">
         <v>3</v>
       </c>
       <c r="L113" s="7" t="s">
-        <v>43</v>
+        <v>611</v>
       </c>
       <c r="M113" s="7" t="s">
-        <v>43</v>
+        <v>611</v>
       </c>
       <c r="N113" s="7" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="O113" s="7" t="s">
-        <v>686</v>
+        <v>682</v>
       </c>
     </row>
     <row r="114" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="10" t="s">
-        <v>687</v>
+        <v>683</v>
       </c>
       <c r="B114" s="11">
         <v>1</v>
@@ -11049,139 +11154,139 @@
         <v>17</v>
       </c>
       <c r="D114" s="11" t="s">
-        <v>659</v>
+        <v>671</v>
       </c>
       <c r="E114" s="11" t="s">
+        <v>684</v>
+      </c>
+      <c r="F114" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="G114" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="H114" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="I114" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="J114" s="11" t="s">
+        <v>686</v>
+      </c>
+      <c r="K114" s="11">
+        <v>3</v>
+      </c>
+      <c r="L114" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="M114" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="N114" s="11" t="s">
+        <v>687</v>
+      </c>
+      <c r="O114" s="11" t="s">
         <v>688</v>
       </c>
-      <c r="F114" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G114" s="11" t="s">
+    </row>
+    <row r="115" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A115" s="6" t="s">
         <v>689</v>
       </c>
-      <c r="H114" s="11" t="s">
+      <c r="B115" s="7">
+        <v>1</v>
+      </c>
+      <c r="C115" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D115" s="7" t="s">
+        <v>671</v>
+      </c>
+      <c r="E115" s="7" t="s">
         <v>690</v>
       </c>
-      <c r="I114" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="J114" s="11" t="s">
+      <c r="F115" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G115" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="H115" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="I115" s="7" t="s">
         <v>691</v>
       </c>
-      <c r="K114" s="11">
-        <v>5</v>
-      </c>
-      <c r="L114" s="11" t="s">
+      <c r="J115" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="K115" s="7">
+        <v>4</v>
+      </c>
+      <c r="L115" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M115" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N115" s="7" t="s">
+        <v>692</v>
+      </c>
+      <c r="O115" s="7" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="116" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A116" s="10" t="s">
+        <v>694</v>
+      </c>
+      <c r="B116" s="11">
+        <v>1</v>
+      </c>
+      <c r="C116" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D116" s="11" t="s">
+        <v>671</v>
+      </c>
+      <c r="E116" s="11" t="s">
+        <v>695</v>
+      </c>
+      <c r="F116" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="G116" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="H116" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="I116" s="11" t="s">
+        <v>696</v>
+      </c>
+      <c r="J116" s="11" t="s">
+        <v>537</v>
+      </c>
+      <c r="K116" s="11">
+        <v>3</v>
+      </c>
+      <c r="L116" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="M114" s="11" t="s">
+      <c r="M116" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="N114" s="11" t="s">
-        <v>692</v>
-      </c>
-      <c r="O114" s="11" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="115" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="12" t="s">
-        <v>694</v>
-      </c>
-      <c r="B115" s="13">
-        <v>1</v>
-      </c>
-      <c r="C115" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D115" s="13" t="s">
-        <v>695</v>
-      </c>
-      <c r="E115" s="13" t="s">
-        <v>696</v>
-      </c>
-      <c r="F115" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="G115" s="13" t="s">
+      <c r="N116" s="11" t="s">
         <v>697</v>
       </c>
-      <c r="H115" s="13" t="s">
+      <c r="O116" s="11" t="s">
         <v>698</v>
-      </c>
-      <c r="I115" s="13" t="s">
-        <v>699</v>
-      </c>
-      <c r="J115" s="13" t="s">
-        <v>700</v>
-      </c>
-      <c r="K115" s="13">
-        <v>3</v>
-      </c>
-      <c r="L115" s="13" t="s">
-        <v>701</v>
-      </c>
-      <c r="M115" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="N115" s="13" t="s">
-        <v>702</v>
-      </c>
-      <c r="O115" s="13" t="s">
-        <v>703</v>
-      </c>
-    </row>
-    <row r="116" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="8" t="s">
-        <v>694</v>
-      </c>
-      <c r="B116" s="9">
-        <v>1</v>
-      </c>
-      <c r="C116" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D116" s="9" t="s">
-        <v>695</v>
-      </c>
-      <c r="E116" s="9" t="s">
-        <v>696</v>
-      </c>
-      <c r="F116" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G116" s="9" t="s">
-        <v>697</v>
-      </c>
-      <c r="H116" s="9" t="s">
-        <v>698</v>
-      </c>
-      <c r="I116" s="9" t="s">
-        <v>699</v>
-      </c>
-      <c r="J116" s="9" t="s">
-        <v>700</v>
-      </c>
-      <c r="K116" s="9">
-        <v>3</v>
-      </c>
-      <c r="L116" s="9" t="s">
-        <v>701</v>
-      </c>
-      <c r="M116" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="N116" s="9" t="s">
-        <v>702</v>
-      </c>
-      <c r="O116" s="9" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="117" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
-        <v>704</v>
+        <v>699</v>
       </c>
       <c r="B117" s="7">
         <v>1</v>
@@ -11190,139 +11295,139 @@
         <v>17</v>
       </c>
       <c r="D117" s="7" t="s">
-        <v>695</v>
+        <v>671</v>
       </c>
       <c r="E117" s="7" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="F117" s="7" t="s">
-        <v>136</v>
+        <v>49</v>
       </c>
       <c r="G117" s="7" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
       <c r="H117" s="7" t="s">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="I117" s="7" t="s">
-        <v>708</v>
+        <v>107</v>
       </c>
       <c r="J117" s="7" t="s">
-        <v>709</v>
+        <v>703</v>
       </c>
       <c r="K117" s="7">
         <v>5</v>
       </c>
       <c r="L117" s="7" t="s">
-        <v>558</v>
+        <v>43</v>
       </c>
       <c r="M117" s="7" t="s">
-        <v>558</v>
+        <v>43</v>
       </c>
       <c r="N117" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="O117" s="7" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="118" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A118" s="14" t="s">
+        <v>706</v>
+      </c>
+      <c r="B118" s="15">
+        <v>1</v>
+      </c>
+      <c r="C118" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D118" s="15" t="s">
+        <v>707</v>
+      </c>
+      <c r="E118" s="15" t="s">
+        <v>708</v>
+      </c>
+      <c r="F118" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="G118" s="15" t="s">
+        <v>709</v>
+      </c>
+      <c r="H118" s="15" t="s">
         <v>710</v>
       </c>
-      <c r="O117" s="7" t="s">
+      <c r="I118" s="15" t="s">
         <v>711</v>
       </c>
-    </row>
-    <row r="118" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A118" s="10" t="s">
+      <c r="J118" s="15" t="s">
         <v>712</v>
       </c>
-      <c r="B118" s="11">
+      <c r="K118" s="15">
+        <v>3</v>
+      </c>
+      <c r="L118" s="15" t="s">
+        <v>713</v>
+      </c>
+      <c r="M118" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="N118" s="15" t="s">
+        <v>714</v>
+      </c>
+      <c r="O118" s="15" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="119" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="8" t="s">
+        <v>706</v>
+      </c>
+      <c r="B119" s="9">
         <v>1</v>
       </c>
-      <c r="C118" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D118" s="11" t="s">
-        <v>695</v>
-      </c>
-      <c r="E118" s="11" t="s">
-        <v>695</v>
-      </c>
-      <c r="F118" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="G118" s="11" t="s">
+      <c r="C119" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D119" s="9" t="s">
+        <v>707</v>
+      </c>
+      <c r="E119" s="9" t="s">
+        <v>708</v>
+      </c>
+      <c r="F119" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G119" s="9" t="s">
+        <v>709</v>
+      </c>
+      <c r="H119" s="9" t="s">
+        <v>710</v>
+      </c>
+      <c r="I119" s="9" t="s">
+        <v>711</v>
+      </c>
+      <c r="J119" s="9" t="s">
+        <v>712</v>
+      </c>
+      <c r="K119" s="9">
+        <v>3</v>
+      </c>
+      <c r="L119" s="9" t="s">
         <v>713</v>
       </c>
-      <c r="H118" s="11" t="s">
+      <c r="M119" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="N119" s="9" t="s">
         <v>714</v>
       </c>
-      <c r="I118" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="J118" s="11" t="s">
-        <v>264</v>
-      </c>
-      <c r="K118" s="11">
-        <v>5</v>
-      </c>
-      <c r="L118" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="M118" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="N118" s="11" t="s">
-        <v>299</v>
-      </c>
-      <c r="O118" s="11" t="s">
+      <c r="O119" s="9" t="s">
         <v>715</v>
-      </c>
-    </row>
-    <row r="119" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A119" s="6" t="s">
-        <v>716</v>
-      </c>
-      <c r="B119" s="7">
-        <v>1</v>
-      </c>
-      <c r="C119" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D119" s="7" t="s">
-        <v>695</v>
-      </c>
-      <c r="E119" s="7" t="s">
-        <v>695</v>
-      </c>
-      <c r="F119" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="G119" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="H119" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="I119" s="7" t="s">
-        <v>717</v>
-      </c>
-      <c r="J119" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="K119" s="7">
-        <v>2</v>
-      </c>
-      <c r="L119" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="M119" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="N119" s="7" t="s">
-        <v>718</v>
-      </c>
-      <c r="O119" s="7" t="s">
-        <v>719</v>
       </c>
     </row>
     <row r="120" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="10" t="s">
-        <v>720</v>
+        <v>716</v>
       </c>
       <c r="B120" s="11">
         <v>1</v>
@@ -11331,34 +11436,34 @@
         <v>17</v>
       </c>
       <c r="D120" s="11" t="s">
-        <v>695</v>
+        <v>707</v>
       </c>
       <c r="E120" s="11" t="s">
-        <v>695</v>
+        <v>717</v>
       </c>
       <c r="F120" s="11" t="s">
-        <v>19</v>
+        <v>136</v>
       </c>
       <c r="G120" s="11" t="s">
-        <v>118</v>
+        <v>718</v>
       </c>
       <c r="H120" s="11" t="s">
-        <v>119</v>
+        <v>719</v>
       </c>
       <c r="I120" s="11" t="s">
-        <v>661</v>
+        <v>720</v>
       </c>
       <c r="J120" s="11" t="s">
         <v>721</v>
       </c>
       <c r="K120" s="11">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L120" s="11" t="s">
-        <v>582</v>
+        <v>566</v>
       </c>
       <c r="M120" s="11" t="s">
-        <v>582</v>
+        <v>566</v>
       </c>
       <c r="N120" s="11" t="s">
         <v>722</v>
@@ -11378,13 +11483,13 @@
         <v>17</v>
       </c>
       <c r="D121" s="7" t="s">
-        <v>695</v>
+        <v>707</v>
       </c>
       <c r="E121" s="7" t="s">
-        <v>695</v>
+        <v>707</v>
       </c>
       <c r="F121" s="7" t="s">
-        <v>136</v>
+        <v>19</v>
       </c>
       <c r="G121" s="7" t="s">
         <v>725</v>
@@ -11393,124 +11498,214 @@
         <v>726</v>
       </c>
       <c r="I121" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="J121" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="K121" s="7">
+        <v>5</v>
+      </c>
+      <c r="L121" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="M121" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="N121" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="O121" s="7" t="s">
         <v>727</v>
       </c>
-      <c r="J121" s="7" t="s">
+    </row>
+    <row r="122" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="B122" s="11">
+        <v>1</v>
+      </c>
+      <c r="C122" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D122" s="11" t="s">
+        <v>707</v>
+      </c>
+      <c r="E122" s="11" t="s">
+        <v>707</v>
+      </c>
+      <c r="F122" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="G122" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="H122" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="I122" s="11" t="s">
+        <v>729</v>
+      </c>
+      <c r="J122" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="K121" s="7">
+      <c r="K122" s="11">
         <v>2</v>
       </c>
-      <c r="L121" s="7" t="s">
+      <c r="L122" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="M121" s="7" t="s">
+      <c r="M122" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="N121" s="7" t="s">
-        <v>544</v>
-      </c>
-      <c r="O121" s="7" t="s">
-        <v>728</v>
-      </c>
-    </row>
-    <row r="122" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A122" s="16" t="s">
-        <v>729</v>
-      </c>
-      <c r="B122" s="17">
+      <c r="N122" s="11" t="s">
+        <v>730</v>
+      </c>
+      <c r="O122" s="11" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="123" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="B123" s="7">
         <v>1</v>
       </c>
-      <c r="C122" s="17" t="s">
+      <c r="C123" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D122" s="17" t="s">
-        <v>695</v>
-      </c>
-      <c r="E122" s="17" t="s">
-        <v>695</v>
-      </c>
-      <c r="F122" s="17" t="s">
+      <c r="D123" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="E123" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="F123" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="G122" s="17" t="s">
-        <v>730</v>
-      </c>
-      <c r="H122" s="17" t="s">
-        <v>731</v>
-      </c>
-      <c r="I122" s="17" t="s">
-        <v>732</v>
-      </c>
-      <c r="J122" s="17" t="s">
+      <c r="G123" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="H123" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="I123" s="7" t="s">
+        <v>673</v>
+      </c>
+      <c r="J123" s="7" t="s">
         <v>733</v>
       </c>
-      <c r="K122" s="17">
+      <c r="K123" s="7">
+        <v>7</v>
+      </c>
+      <c r="L123" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="M123" s="7" t="s">
+        <v>594</v>
+      </c>
+      <c r="N123" s="7" t="s">
+        <v>734</v>
+      </c>
+      <c r="O123" s="7" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="124" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="10" t="s">
+        <v>736</v>
+      </c>
+      <c r="B124" s="11">
+        <v>1</v>
+      </c>
+      <c r="C124" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D124" s="11" t="s">
+        <v>707</v>
+      </c>
+      <c r="E124" s="11" t="s">
+        <v>707</v>
+      </c>
+      <c r="F124" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="G124" s="11" t="s">
+        <v>737</v>
+      </c>
+      <c r="H124" s="11" t="s">
+        <v>738</v>
+      </c>
+      <c r="I124" s="11" t="s">
+        <v>739</v>
+      </c>
+      <c r="J124" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="K124" s="11">
+        <v>2</v>
+      </c>
+      <c r="L124" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="M124" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="N124" s="11" t="s">
+        <v>552</v>
+      </c>
+      <c r="O124" s="11" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="125" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="16" t="s">
+        <v>741</v>
+      </c>
+      <c r="B125" s="17">
+        <v>1</v>
+      </c>
+      <c r="C125" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D125" s="17" t="s">
+        <v>707</v>
+      </c>
+      <c r="E125" s="17" t="s">
+        <v>707</v>
+      </c>
+      <c r="F125" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="G125" s="17" t="s">
+        <v>742</v>
+      </c>
+      <c r="H125" s="17" t="s">
+        <v>743</v>
+      </c>
+      <c r="I125" s="17" t="s">
+        <v>744</v>
+      </c>
+      <c r="J125" s="17" t="s">
+        <v>745</v>
+      </c>
+      <c r="K125" s="17">
         <v>3</v>
       </c>
-      <c r="L122" s="17" t="s">
+      <c r="L125" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="M122" s="17" t="s">
+      <c r="M125" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="N122" s="17" t="s">
+      <c r="N125" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="O122" s="17" t="s">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="123" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="1"/>
-      <c r="B123" s="1"/>
-      <c r="C123" s="1"/>
-      <c r="D123" s="1"/>
-      <c r="E123" s="1"/>
-      <c r="F123" s="1"/>
-      <c r="G123" s="1"/>
-      <c r="H123" s="1"/>
-      <c r="I123" s="1"/>
-      <c r="J123" s="1"/>
-      <c r="K123" s="1"/>
-      <c r="L123" s="1"/>
-      <c r="M123" s="1"/>
-      <c r="N123" s="1"/>
-      <c r="O123" s="1"/>
-    </row>
-    <row r="124" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="1"/>
-      <c r="B124" s="1"/>
-      <c r="C124" s="1"/>
-      <c r="D124" s="1"/>
-      <c r="E124" s="1"/>
-      <c r="F124" s="1"/>
-      <c r="G124" s="1"/>
-      <c r="H124" s="1"/>
-      <c r="I124" s="1"/>
-      <c r="J124" s="1"/>
-      <c r="K124" s="1"/>
-      <c r="L124" s="1"/>
-      <c r="M124" s="1"/>
-      <c r="N124" s="1"/>
-      <c r="O124" s="1"/>
-    </row>
-    <row r="125" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A125" s="1"/>
-      <c r="B125" s="1"/>
-      <c r="C125" s="1"/>
-      <c r="D125" s="1"/>
-      <c r="E125" s="1"/>
-      <c r="F125" s="1"/>
-      <c r="G125" s="1"/>
-      <c r="H125" s="1"/>
-      <c r="I125" s="1"/>
-      <c r="J125" s="1"/>
-      <c r="K125" s="1"/>
-      <c r="L125" s="1"/>
-      <c r="M125" s="1"/>
-      <c r="N125" s="1"/>
-      <c r="O125" s="1"/>
+      <c r="O125" s="17" t="s">
+        <v>746</v>
+      </c>
     </row>
     <row r="126" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1"/>
@@ -14860,6 +15055,57 @@
       <c r="M322" s="1"/>
       <c r="N322" s="1"/>
       <c r="O322" s="1"/>
+    </row>
+    <row r="323" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A323" s="1"/>
+      <c r="B323" s="1"/>
+      <c r="C323" s="1"/>
+      <c r="D323" s="1"/>
+      <c r="E323" s="1"/>
+      <c r="F323" s="1"/>
+      <c r="G323" s="1"/>
+      <c r="H323" s="1"/>
+      <c r="I323" s="1"/>
+      <c r="J323" s="1"/>
+      <c r="K323" s="1"/>
+      <c r="L323" s="1"/>
+      <c r="M323" s="1"/>
+      <c r="N323" s="1"/>
+      <c r="O323" s="1"/>
+    </row>
+    <row r="324" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A324" s="1"/>
+      <c r="B324" s="1"/>
+      <c r="C324" s="1"/>
+      <c r="D324" s="1"/>
+      <c r="E324" s="1"/>
+      <c r="F324" s="1"/>
+      <c r="G324" s="1"/>
+      <c r="H324" s="1"/>
+      <c r="I324" s="1"/>
+      <c r="J324" s="1"/>
+      <c r="K324" s="1"/>
+      <c r="L324" s="1"/>
+      <c r="M324" s="1"/>
+      <c r="N324" s="1"/>
+      <c r="O324" s="1"/>
+    </row>
+    <row r="325" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A325" s="1"/>
+      <c r="B325" s="1"/>
+      <c r="C325" s="1"/>
+      <c r="D325" s="1"/>
+      <c r="E325" s="1"/>
+      <c r="F325" s="1"/>
+      <c r="G325" s="1"/>
+      <c r="H325" s="1"/>
+      <c r="I325" s="1"/>
+      <c r="J325" s="1"/>
+      <c r="K325" s="1"/>
+      <c r="L325" s="1"/>
+      <c r="M325" s="1"/>
+      <c r="N325" s="1"/>
+      <c r="O325" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -14986,9 +15232,12 @@
     <hyperlink ref="O120" r:id="rId118"/>
     <hyperlink ref="O121" r:id="rId119"/>
     <hyperlink ref="O122" r:id="rId120"/>
+    <hyperlink ref="O123" r:id="rId121"/>
+    <hyperlink ref="O124" r:id="rId122"/>
+    <hyperlink ref="O125" r:id="rId123"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId122"/>
+  <legacyDrawing r:id="rId125"/>
 </worksheet>
 </file>
</xml_diff>